<commit_message>
Curva S actualizada 2026-09-05 18:13 Chile
</commit_message>
<xml_diff>
--- a/data/50001569 -  EUROHINCA.xlsx
+++ b/data/50001569 -  EUROHINCA.xlsx
@@ -1966,7 +1966,7 @@
         <v>46206.67847994213</v>
       </c>
       <c r="D4" s="5">
-        <v>46206.6784915162</v>
+        <v>46270.90847643519</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>24</v>
@@ -2886,7 +2886,7 @@
         <v>46206.76952165509</v>
       </c>
       <c r="D20" s="5">
-        <v>46206.76953472222</v>
+        <v>46270.90897929398</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>69</v>
@@ -3189,7 +3189,7 @@
         <v>46260.881508125</v>
       </c>
       <c r="D25" s="9">
-        <v>46260.881520740746</v>
+        <v>46270.90921540509</v>
       </c>
       <c r="E25" s="10" t="s">
         <v>86</v>
@@ -3630,7 +3630,7 @@
       </c>
       <c r="C32" s="6"/>
       <c r="D32" s="5">
-        <v>46251.584816585644</v>
+        <v>46270.9090384375</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>111</v>
@@ -6320,7 +6320,7 @@
       </c>
       <c r="C78" s="6"/>
       <c r="D78" s="5">
-        <v>46206.67094998843</v>
+        <v>46270.9214584838</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>206</v>

</xml_diff>